<commit_message>
Add Day05 contacts app and update study handoff notes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/學習進度打卡表.xlsx
+++ b/學習進度打卡表.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\林芯緹\Desktop\Learn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF05909-C683-4779-846A-EA350017719A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545151EA-F394-4841-A5B5-045504C7E78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="279">
   <si>
     <t>C# .NET 學習進度打卡表</t>
   </si>
@@ -892,6 +892,10 @@
     <t>缺字串處理工具</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
+  <si>
+    <t>✔</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
@@ -902,7 +906,7 @@
     <numFmt numFmtId="177" formatCode="0.0%"/>
     <numFmt numFmtId="178" formatCode="0.0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -975,6 +979,11 @@
       <charset val="136"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1036,7 +1045,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1114,6 +1123,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1508,7 +1520,7 @@
       </c>
       <c r="C11" s="24">
         <f>SUM(每日打卡!$J$2:$J$101)</f>
-        <v>7</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="12" spans="2:4">
@@ -1992,14 +2004,16 @@
         <f>WORKDAY(總覽!$C$4,A5-1)</f>
         <v>46296</v>
       </c>
-      <c r="H5" s="19" t="s">
-        <v>52</v>
+      <c r="H5" s="31" t="s">
+        <v>278</v>
       </c>
       <c r="I5" s="17">
         <f>總覽!$C$5</f>
         <v>3.5</v>
       </c>
-      <c r="J5" s="19"/>
+      <c r="J5" s="19">
+        <v>1.5</v>
+      </c>
       <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:11">

</xml_diff>

<commit_message>
Add Day06 contacts interface refactor and virtual experiment
- Day06_Contacts: extract IContactBook interface and ContactBook implementation; menu now depends only on the interface
- Day06_Virtual: virtual/override experiment
- Update study handoff notes and progress sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/學習進度打卡表.xlsx
+++ b/學習進度打卡表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\林芯緹\Desktop\Learn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{545151EA-F394-4841-A5B5-045504C7E78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1469646-49B0-4071-93FB-5E1E22556B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="總覽" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="281">
   <si>
     <t>C# .NET 學習進度打卡表</t>
   </si>
@@ -256,9 +256,6 @@
     <t>通訊錄(記憶體版)</t>
   </si>
   <si>
-    <t>interface、繼承、多型</t>
-  </si>
-  <si>
     <t>為通訊錄抽出介面</t>
   </si>
   <si>
@@ -894,6 +891,100 @@
   </si>
   <si>
     <t>✔</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>【C#】複習＋通訊錄實作：class 設計、建構子驗證、例外處理、while/switch 選單</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <t>interface、繼承、多型</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>為什麼 ContactBook 裡不能有 Console.WriteLine?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+名片盒不會開口說話。說話是選單的工作,這樣換一個名片盒時,說話的部分不用重寫。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>IContactBook book = new ContactBook(); 左邊為什麼寫介面?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+左邊寫介面,以後只要換右邊,選單其他地方都不用改。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>if (c) 在 JS 可以,C# 為什麼不行?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+C# 的 if 括號裡只接受 bool,不會自動把物件轉成 true/false。所以要自己寫出比較:c != null。
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>null 和空清單差在哪?</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Microsoft JhengHei"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve">
+null是手上沒有盒子，空清單是手上有盒子,但裡面 0 張</t>
+    </r>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
 </sst>
@@ -906,7 +997,7 @@
     <numFmt numFmtId="177" formatCode="0.0%"/>
     <numFmt numFmtId="178" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -983,6 +1074,13 @@
       <sz val="10"/>
       <name val="Segoe UI Symbol"/>
       <family val="3"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Microsoft JhengHei"/>
+      <family val="2"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1119,13 +1217,13 @@
     <xf numFmtId="176" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -1493,7 +1591,7 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF(每日打卡!$H$2:$H$101,"✔")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="2:4">
@@ -1511,7 +1609,7 @@
       </c>
       <c r="C10" s="23">
         <f>IFERROR(C8/C9,0)</f>
-        <v>0.04</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="11" spans="2:4">
@@ -1520,7 +1618,7 @@
       </c>
       <c r="C11" s="24">
         <f>SUM(每日打卡!$J$2:$J$101)</f>
-        <v>8.5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="2:4">
@@ -1581,7 +1679,7 @@
       </c>
       <c r="D18" s="11">
         <f>COUNTIFS(每日打卡!$D$2:$D$101,B18,每日打卡!$H$2:$H$101,"✔")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E18" s="11">
         <f>COUNTIF(每日打卡!$D$2:$D$101,B18)</f>
@@ -1589,7 +1687,7 @@
       </c>
       <c r="F18" s="12">
         <f t="shared" ref="F18:F25" si="0">IFERROR(D18/E18,0)</f>
-        <v>0.4</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="19" spans="2:7">
@@ -1738,64 +1836,64 @@
       </c>
     </row>
     <row r="28" spans="2:7" ht="30" customHeight="1">
-      <c r="B28" s="29" t="s">
+      <c r="B28" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30"/>
-      <c r="E28" s="30"/>
-      <c r="F28" s="30"/>
-      <c r="G28" s="30"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
+      <c r="G28" s="31"/>
     </row>
     <row r="29" spans="2:7" ht="30" customHeight="1">
-      <c r="B29" s="29" t="s">
+      <c r="B29" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="D29" s="30"/>
-      <c r="E29" s="30"/>
-      <c r="F29" s="30"/>
-      <c r="G29" s="30"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
+      <c r="G29" s="31"/>
     </row>
     <row r="30" spans="2:7" ht="30" customHeight="1">
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="30" t="s">
         <v>35</v>
       </c>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30"/>
-      <c r="E30" s="30"/>
-      <c r="F30" s="30"/>
-      <c r="G30" s="30"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
+      <c r="E30" s="31"/>
+      <c r="F30" s="31"/>
+      <c r="G30" s="31"/>
     </row>
     <row r="31" spans="2:7" ht="30" customHeight="1">
-      <c r="B31" s="29" t="s">
+      <c r="B31" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30"/>
-      <c r="E31" s="30"/>
-      <c r="F31" s="30"/>
-      <c r="G31" s="30"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="31"/>
+      <c r="F31" s="31"/>
+      <c r="G31" s="31"/>
     </row>
     <row r="32" spans="2:7" ht="30" customHeight="1">
-      <c r="B32" s="29" t="s">
+      <c r="B32" s="30" t="s">
         <v>37</v>
       </c>
-      <c r="C32" s="30"/>
-      <c r="D32" s="30"/>
-      <c r="E32" s="30"/>
-      <c r="F32" s="30"/>
-      <c r="G32" s="30"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
+      <c r="E32" s="31"/>
+      <c r="F32" s="31"/>
+      <c r="G32" s="31"/>
     </row>
     <row r="33" spans="2:7" ht="30" customHeight="1">
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C33" s="30"/>
-      <c r="D33" s="30"/>
-      <c r="E33" s="30"/>
-      <c r="F33" s="30"/>
-      <c r="G33" s="30"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
+      <c r="E33" s="31"/>
+      <c r="F33" s="31"/>
+      <c r="G33" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1978,7 +2076,7 @@
         <v>3</v>
       </c>
       <c r="K4" s="20" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2004,8 +2102,8 @@
         <f>WORKDAY(總覽!$C$4,A5-1)</f>
         <v>46296</v>
       </c>
-      <c r="H5" s="31" t="s">
-        <v>278</v>
+      <c r="H5" s="29" t="s">
+        <v>277</v>
       </c>
       <c r="I5" s="17">
         <f>總覽!$C$5</f>
@@ -2039,15 +2137,21 @@
         <f>WORKDAY(總覽!$C$4,A6-1)</f>
         <v>46297</v>
       </c>
-      <c r="H6" s="19"/>
+      <c r="H6" s="19" t="s">
+        <v>52</v>
+      </c>
       <c r="I6" s="17">
         <f>總覽!$C$5</f>
         <v>3.5</v>
       </c>
-      <c r="J6" s="19"/>
-      <c r="K6" s="20"/>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="J6" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="108">
       <c r="A7" s="13">
         <v>6</v>
       </c>
@@ -2061,22 +2165,28 @@
         <v>16</v>
       </c>
       <c r="E7" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="F7" s="14" t="s">
         <v>66</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>67</v>
       </c>
       <c r="G7" s="26">
         <f>WORKDAY(總覽!$C$4,A7-1)</f>
         <v>46300</v>
       </c>
-      <c r="H7" s="15"/>
+      <c r="H7" s="15" t="s">
+        <v>52</v>
+      </c>
       <c r="I7" s="13">
         <f>總覽!$C$5</f>
         <v>3.5</v>
       </c>
-      <c r="J7" s="15"/>
-      <c r="K7" s="16"/>
+      <c r="J7" s="15">
+        <v>3</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>280</v>
+      </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="17">
@@ -2092,10 +2202,10 @@
         <v>16</v>
       </c>
       <c r="E8" s="18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F8" s="18" t="s">
         <v>68</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>69</v>
       </c>
       <c r="G8" s="27">
         <f>WORKDAY(總覽!$C$4,A8-1)</f>
@@ -2123,10 +2233,10 @@
         <v>16</v>
       </c>
       <c r="E9" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>70</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>71</v>
       </c>
       <c r="G9" s="27">
         <f>WORKDAY(總覽!$C$4,A9-1)</f>
@@ -2154,10 +2264,10 @@
         <v>16</v>
       </c>
       <c r="E10" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" s="18" t="s">
         <v>72</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>73</v>
       </c>
       <c r="G10" s="27">
         <f>WORKDAY(總覽!$C$4,A10-1)</f>
@@ -2185,10 +2295,10 @@
         <v>16</v>
       </c>
       <c r="E11" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>74</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>75</v>
       </c>
       <c r="G11" s="27">
         <f>WORKDAY(總覽!$C$4,A11-1)</f>
@@ -2216,10 +2326,10 @@
         <v>18</v>
       </c>
       <c r="E12" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F12" s="14" t="s">
         <v>76</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>77</v>
       </c>
       <c r="G12" s="26">
         <f>WORKDAY(總覽!$C$4,A12-1)</f>
@@ -2247,10 +2357,10 @@
         <v>18</v>
       </c>
       <c r="E13" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>78</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>79</v>
       </c>
       <c r="G13" s="27">
         <f>WORKDAY(總覽!$C$4,A13-1)</f>
@@ -2278,10 +2388,10 @@
         <v>18</v>
       </c>
       <c r="E14" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>80</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>81</v>
       </c>
       <c r="G14" s="27">
         <f>WORKDAY(總覽!$C$4,A14-1)</f>
@@ -2309,10 +2419,10 @@
         <v>18</v>
       </c>
       <c r="E15" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>82</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>83</v>
       </c>
       <c r="G15" s="27">
         <f>WORKDAY(總覽!$C$4,A15-1)</f>
@@ -2340,10 +2450,10 @@
         <v>18</v>
       </c>
       <c r="E16" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="18" t="s">
         <v>84</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>85</v>
       </c>
       <c r="G16" s="27">
         <f>WORKDAY(總覽!$C$4,A16-1)</f>
@@ -2371,10 +2481,10 @@
         <v>18</v>
       </c>
       <c r="E17" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="14" t="s">
         <v>86</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>87</v>
       </c>
       <c r="G17" s="26">
         <f>WORKDAY(總覽!$C$4,A17-1)</f>
@@ -2402,10 +2512,10 @@
         <v>18</v>
       </c>
       <c r="E18" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>88</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>89</v>
       </c>
       <c r="G18" s="27">
         <f>WORKDAY(總覽!$C$4,A18-1)</f>
@@ -2433,10 +2543,10 @@
         <v>18</v>
       </c>
       <c r="E19" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>90</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>91</v>
       </c>
       <c r="G19" s="27">
         <f>WORKDAY(總覽!$C$4,A19-1)</f>
@@ -2464,10 +2574,10 @@
         <v>18</v>
       </c>
       <c r="E20" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="F20" s="18" t="s">
         <v>92</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>93</v>
       </c>
       <c r="G20" s="27">
         <f>WORKDAY(總覽!$C$4,A20-1)</f>
@@ -2495,10 +2605,10 @@
         <v>18</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G21" s="27">
         <f>WORKDAY(總覽!$C$4,A21-1)</f>
@@ -2526,10 +2636,10 @@
         <v>20</v>
       </c>
       <c r="E22" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="14" t="s">
         <v>95</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>96</v>
       </c>
       <c r="G22" s="26">
         <f>WORKDAY(總覽!$C$4,A22-1)</f>
@@ -2557,10 +2667,10 @@
         <v>20</v>
       </c>
       <c r="E23" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>97</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>98</v>
       </c>
       <c r="G23" s="27">
         <f>WORKDAY(總覽!$C$4,A23-1)</f>
@@ -2588,10 +2698,10 @@
         <v>20</v>
       </c>
       <c r="E24" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>99</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>100</v>
       </c>
       <c r="G24" s="27">
         <f>WORKDAY(總覽!$C$4,A24-1)</f>
@@ -2619,10 +2729,10 @@
         <v>20</v>
       </c>
       <c r="E25" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>101</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>102</v>
       </c>
       <c r="G25" s="27">
         <f>WORKDAY(總覽!$C$4,A25-1)</f>
@@ -2650,10 +2760,10 @@
         <v>20</v>
       </c>
       <c r="E26" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="18" t="s">
         <v>103</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>104</v>
       </c>
       <c r="G26" s="27">
         <f>WORKDAY(總覽!$C$4,A26-1)</f>
@@ -2681,10 +2791,10 @@
         <v>20</v>
       </c>
       <c r="E27" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" s="14" t="s">
         <v>105</v>
-      </c>
-      <c r="F27" s="14" t="s">
-        <v>106</v>
       </c>
       <c r="G27" s="26">
         <f>WORKDAY(總覽!$C$4,A27-1)</f>
@@ -2712,10 +2822,10 @@
         <v>20</v>
       </c>
       <c r="E28" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="18" t="s">
         <v>107</v>
-      </c>
-      <c r="F28" s="18" t="s">
-        <v>108</v>
       </c>
       <c r="G28" s="27">
         <f>WORKDAY(總覽!$C$4,A28-1)</f>
@@ -2743,10 +2853,10 @@
         <v>20</v>
       </c>
       <c r="E29" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="F29" s="18" t="s">
         <v>109</v>
-      </c>
-      <c r="F29" s="18" t="s">
-        <v>110</v>
       </c>
       <c r="G29" s="27">
         <f>WORKDAY(總覽!$C$4,A29-1)</f>
@@ -2774,10 +2884,10 @@
         <v>20</v>
       </c>
       <c r="E30" s="18" t="s">
+        <v>110</v>
+      </c>
+      <c r="F30" s="18" t="s">
         <v>111</v>
-      </c>
-      <c r="F30" s="18" t="s">
-        <v>112</v>
       </c>
       <c r="G30" s="27">
         <f>WORKDAY(總覽!$C$4,A30-1)</f>
@@ -2805,10 +2915,10 @@
         <v>20</v>
       </c>
       <c r="E31" s="18" t="s">
+        <v>112</v>
+      </c>
+      <c r="F31" s="18" t="s">
         <v>113</v>
-      </c>
-      <c r="F31" s="18" t="s">
-        <v>114</v>
       </c>
       <c r="G31" s="27">
         <f>WORKDAY(總覽!$C$4,A31-1)</f>
@@ -2836,10 +2946,10 @@
         <v>20</v>
       </c>
       <c r="E32" s="14" t="s">
+        <v>114</v>
+      </c>
+      <c r="F32" s="14" t="s">
         <v>115</v>
-      </c>
-      <c r="F32" s="14" t="s">
-        <v>116</v>
       </c>
       <c r="G32" s="26">
         <f>WORKDAY(總覽!$C$4,A32-1)</f>
@@ -2867,10 +2977,10 @@
         <v>20</v>
       </c>
       <c r="E33" s="18" t="s">
+        <v>116</v>
+      </c>
+      <c r="F33" s="18" t="s">
         <v>117</v>
-      </c>
-      <c r="F33" s="18" t="s">
-        <v>118</v>
       </c>
       <c r="G33" s="27">
         <f>WORKDAY(總覽!$C$4,A33-1)</f>
@@ -2898,10 +3008,10 @@
         <v>20</v>
       </c>
       <c r="E34" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="F34" s="18" t="s">
         <v>119</v>
-      </c>
-      <c r="F34" s="18" t="s">
-        <v>120</v>
       </c>
       <c r="G34" s="27">
         <f>WORKDAY(總覽!$C$4,A34-1)</f>
@@ -2929,10 +3039,10 @@
         <v>20</v>
       </c>
       <c r="E35" s="18" t="s">
+        <v>120</v>
+      </c>
+      <c r="F35" s="18" t="s">
         <v>121</v>
-      </c>
-      <c r="F35" s="18" t="s">
-        <v>122</v>
       </c>
       <c r="G35" s="27">
         <f>WORKDAY(總覽!$C$4,A35-1)</f>
@@ -2960,10 +3070,10 @@
         <v>20</v>
       </c>
       <c r="E36" s="18" t="s">
+        <v>122</v>
+      </c>
+      <c r="F36" s="18" t="s">
         <v>123</v>
-      </c>
-      <c r="F36" s="18" t="s">
-        <v>124</v>
       </c>
       <c r="G36" s="27">
         <f>WORKDAY(總覽!$C$4,A36-1)</f>
@@ -2991,10 +3101,10 @@
         <v>22</v>
       </c>
       <c r="E37" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="F37" s="14" t="s">
         <v>125</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>126</v>
       </c>
       <c r="G37" s="26">
         <f>WORKDAY(總覽!$C$4,A37-1)</f>
@@ -3022,10 +3132,10 @@
         <v>22</v>
       </c>
       <c r="E38" s="18" t="s">
+        <v>126</v>
+      </c>
+      <c r="F38" s="18" t="s">
         <v>127</v>
-      </c>
-      <c r="F38" s="18" t="s">
-        <v>128</v>
       </c>
       <c r="G38" s="27">
         <f>WORKDAY(總覽!$C$4,A38-1)</f>
@@ -3053,10 +3163,10 @@
         <v>22</v>
       </c>
       <c r="E39" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="F39" s="18" t="s">
         <v>129</v>
-      </c>
-      <c r="F39" s="18" t="s">
-        <v>130</v>
       </c>
       <c r="G39" s="27">
         <f>WORKDAY(總覽!$C$4,A39-1)</f>
@@ -3084,10 +3194,10 @@
         <v>22</v>
       </c>
       <c r="E40" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="F40" s="18" t="s">
         <v>131</v>
-      </c>
-      <c r="F40" s="18" t="s">
-        <v>132</v>
       </c>
       <c r="G40" s="27">
         <f>WORKDAY(總覽!$C$4,A40-1)</f>
@@ -3115,10 +3225,10 @@
         <v>22</v>
       </c>
       <c r="E41" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="F41" s="18" t="s">
         <v>133</v>
-      </c>
-      <c r="F41" s="18" t="s">
-        <v>134</v>
       </c>
       <c r="G41" s="27">
         <f>WORKDAY(總覽!$C$4,A41-1)</f>
@@ -3146,10 +3256,10 @@
         <v>22</v>
       </c>
       <c r="E42" s="14" t="s">
+        <v>134</v>
+      </c>
+      <c r="F42" s="14" t="s">
         <v>135</v>
-      </c>
-      <c r="F42" s="14" t="s">
-        <v>136</v>
       </c>
       <c r="G42" s="26">
         <f>WORKDAY(總覽!$C$4,A42-1)</f>
@@ -3177,10 +3287,10 @@
         <v>22</v>
       </c>
       <c r="E43" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="F43" s="18" t="s">
         <v>137</v>
-      </c>
-      <c r="F43" s="18" t="s">
-        <v>138</v>
       </c>
       <c r="G43" s="27">
         <f>WORKDAY(總覽!$C$4,A43-1)</f>
@@ -3208,10 +3318,10 @@
         <v>22</v>
       </c>
       <c r="E44" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="F44" s="18" t="s">
         <v>139</v>
-      </c>
-      <c r="F44" s="18" t="s">
-        <v>140</v>
       </c>
       <c r="G44" s="27">
         <f>WORKDAY(總覽!$C$4,A44-1)</f>
@@ -3239,10 +3349,10 @@
         <v>22</v>
       </c>
       <c r="E45" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="F45" s="18" t="s">
         <v>141</v>
-      </c>
-      <c r="F45" s="18" t="s">
-        <v>142</v>
       </c>
       <c r="G45" s="27">
         <f>WORKDAY(總覽!$C$4,A45-1)</f>
@@ -3270,10 +3380,10 @@
         <v>22</v>
       </c>
       <c r="E46" s="18" t="s">
+        <v>142</v>
+      </c>
+      <c r="F46" s="18" t="s">
         <v>143</v>
-      </c>
-      <c r="F46" s="18" t="s">
-        <v>144</v>
       </c>
       <c r="G46" s="27">
         <f>WORKDAY(總覽!$C$4,A46-1)</f>
@@ -3301,10 +3411,10 @@
         <v>24</v>
       </c>
       <c r="E47" s="14" t="s">
+        <v>144</v>
+      </c>
+      <c r="F47" s="14" t="s">
         <v>145</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>146</v>
       </c>
       <c r="G47" s="26">
         <f>WORKDAY(總覽!$C$4,A47-1)</f>
@@ -3332,10 +3442,10 @@
         <v>24</v>
       </c>
       <c r="E48" s="18" t="s">
+        <v>146</v>
+      </c>
+      <c r="F48" s="18" t="s">
         <v>147</v>
-      </c>
-      <c r="F48" s="18" t="s">
-        <v>148</v>
       </c>
       <c r="G48" s="27">
         <f>WORKDAY(總覽!$C$4,A48-1)</f>
@@ -3363,10 +3473,10 @@
         <v>24</v>
       </c>
       <c r="E49" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="F49" s="18" t="s">
         <v>149</v>
-      </c>
-      <c r="F49" s="18" t="s">
-        <v>150</v>
       </c>
       <c r="G49" s="27">
         <f>WORKDAY(總覽!$C$4,A49-1)</f>
@@ -3394,10 +3504,10 @@
         <v>24</v>
       </c>
       <c r="E50" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="F50" s="18" t="s">
         <v>151</v>
-      </c>
-      <c r="F50" s="18" t="s">
-        <v>152</v>
       </c>
       <c r="G50" s="27">
         <f>WORKDAY(總覽!$C$4,A50-1)</f>
@@ -3425,10 +3535,10 @@
         <v>24</v>
       </c>
       <c r="E51" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="F51" s="18" t="s">
         <v>153</v>
-      </c>
-      <c r="F51" s="18" t="s">
-        <v>154</v>
       </c>
       <c r="G51" s="27">
         <f>WORKDAY(總覽!$C$4,A51-1)</f>
@@ -3456,10 +3566,10 @@
         <v>24</v>
       </c>
       <c r="E52" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="F52" s="14" t="s">
         <v>155</v>
-      </c>
-      <c r="F52" s="14" t="s">
-        <v>156</v>
       </c>
       <c r="G52" s="26">
         <f>WORKDAY(總覽!$C$4,A52-1)</f>
@@ -3487,10 +3597,10 @@
         <v>24</v>
       </c>
       <c r="E53" s="18" t="s">
+        <v>156</v>
+      </c>
+      <c r="F53" s="18" t="s">
         <v>157</v>
-      </c>
-      <c r="F53" s="18" t="s">
-        <v>158</v>
       </c>
       <c r="G53" s="27">
         <f>WORKDAY(總覽!$C$4,A53-1)</f>
@@ -3518,10 +3628,10 @@
         <v>24</v>
       </c>
       <c r="E54" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="F54" s="18" t="s">
         <v>159</v>
-      </c>
-      <c r="F54" s="18" t="s">
-        <v>160</v>
       </c>
       <c r="G54" s="27">
         <f>WORKDAY(總覽!$C$4,A54-1)</f>
@@ -3549,10 +3659,10 @@
         <v>24</v>
       </c>
       <c r="E55" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="F55" s="18" t="s">
         <v>161</v>
-      </c>
-      <c r="F55" s="18" t="s">
-        <v>162</v>
       </c>
       <c r="G55" s="27">
         <f>WORKDAY(總覽!$C$4,A55-1)</f>
@@ -3580,10 +3690,10 @@
         <v>24</v>
       </c>
       <c r="E56" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="F56" s="18" t="s">
         <v>163</v>
-      </c>
-      <c r="F56" s="18" t="s">
-        <v>164</v>
       </c>
       <c r="G56" s="27">
         <f>WORKDAY(總覽!$C$4,A56-1)</f>
@@ -3611,10 +3721,10 @@
         <v>26</v>
       </c>
       <c r="E57" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="F57" s="14" t="s">
         <v>165</v>
-      </c>
-      <c r="F57" s="14" t="s">
-        <v>166</v>
       </c>
       <c r="G57" s="26">
         <f>WORKDAY(總覽!$C$4,A57-1)</f>
@@ -3642,10 +3752,10 @@
         <v>26</v>
       </c>
       <c r="E58" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="F58" s="18" t="s">
         <v>167</v>
-      </c>
-      <c r="F58" s="18" t="s">
-        <v>168</v>
       </c>
       <c r="G58" s="27">
         <f>WORKDAY(總覽!$C$4,A58-1)</f>
@@ -3673,10 +3783,10 @@
         <v>26</v>
       </c>
       <c r="E59" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="F59" s="18" t="s">
         <v>169</v>
-      </c>
-      <c r="F59" s="18" t="s">
-        <v>170</v>
       </c>
       <c r="G59" s="27">
         <f>WORKDAY(總覽!$C$4,A59-1)</f>
@@ -3704,10 +3814,10 @@
         <v>26</v>
       </c>
       <c r="E60" s="18" t="s">
+        <v>170</v>
+      </c>
+      <c r="F60" s="18" t="s">
         <v>171</v>
-      </c>
-      <c r="F60" s="18" t="s">
-        <v>172</v>
       </c>
       <c r="G60" s="27">
         <f>WORKDAY(總覽!$C$4,A60-1)</f>
@@ -3735,10 +3845,10 @@
         <v>26</v>
       </c>
       <c r="E61" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="F61" s="18" t="s">
         <v>173</v>
-      </c>
-      <c r="F61" s="18" t="s">
-        <v>174</v>
       </c>
       <c r="G61" s="27">
         <f>WORKDAY(總覽!$C$4,A61-1)</f>
@@ -3766,10 +3876,10 @@
         <v>26</v>
       </c>
       <c r="E62" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="F62" s="14" t="s">
         <v>175</v>
-      </c>
-      <c r="F62" s="14" t="s">
-        <v>176</v>
       </c>
       <c r="G62" s="26">
         <f>WORKDAY(總覽!$C$4,A62-1)</f>
@@ -3797,10 +3907,10 @@
         <v>26</v>
       </c>
       <c r="E63" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="F63" s="18" t="s">
         <v>177</v>
-      </c>
-      <c r="F63" s="18" t="s">
-        <v>178</v>
       </c>
       <c r="G63" s="27">
         <f>WORKDAY(總覽!$C$4,A63-1)</f>
@@ -3828,10 +3938,10 @@
         <v>26</v>
       </c>
       <c r="E64" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="F64" s="18" t="s">
         <v>179</v>
-      </c>
-      <c r="F64" s="18" t="s">
-        <v>180</v>
       </c>
       <c r="G64" s="27">
         <f>WORKDAY(總覽!$C$4,A64-1)</f>
@@ -3859,10 +3969,10 @@
         <v>26</v>
       </c>
       <c r="E65" s="18" t="s">
+        <v>180</v>
+      </c>
+      <c r="F65" s="18" t="s">
         <v>181</v>
-      </c>
-      <c r="F65" s="18" t="s">
-        <v>182</v>
       </c>
       <c r="G65" s="27">
         <f>WORKDAY(總覽!$C$4,A65-1)</f>
@@ -3890,10 +4000,10 @@
         <v>26</v>
       </c>
       <c r="E66" s="18" t="s">
+        <v>182</v>
+      </c>
+      <c r="F66" s="18" t="s">
         <v>183</v>
-      </c>
-      <c r="F66" s="18" t="s">
-        <v>184</v>
       </c>
       <c r="G66" s="27">
         <f>WORKDAY(總覽!$C$4,A66-1)</f>
@@ -3921,10 +4031,10 @@
         <v>28</v>
       </c>
       <c r="E67" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="F67" s="14" t="s">
         <v>185</v>
-      </c>
-      <c r="F67" s="14" t="s">
-        <v>186</v>
       </c>
       <c r="G67" s="26">
         <f>WORKDAY(總覽!$C$4,A67-1)</f>
@@ -3952,10 +4062,10 @@
         <v>28</v>
       </c>
       <c r="E68" s="18" t="s">
+        <v>186</v>
+      </c>
+      <c r="F68" s="18" t="s">
         <v>187</v>
-      </c>
-      <c r="F68" s="18" t="s">
-        <v>188</v>
       </c>
       <c r="G68" s="27">
         <f>WORKDAY(總覽!$C$4,A68-1)</f>
@@ -3983,10 +4093,10 @@
         <v>28</v>
       </c>
       <c r="E69" s="18" t="s">
+        <v>188</v>
+      </c>
+      <c r="F69" s="18" t="s">
         <v>189</v>
-      </c>
-      <c r="F69" s="18" t="s">
-        <v>190</v>
       </c>
       <c r="G69" s="27">
         <f>WORKDAY(總覽!$C$4,A69-1)</f>
@@ -4014,10 +4124,10 @@
         <v>28</v>
       </c>
       <c r="E70" s="18" t="s">
+        <v>190</v>
+      </c>
+      <c r="F70" s="18" t="s">
         <v>191</v>
-      </c>
-      <c r="F70" s="18" t="s">
-        <v>192</v>
       </c>
       <c r="G70" s="27">
         <f>WORKDAY(總覽!$C$4,A70-1)</f>
@@ -4045,10 +4155,10 @@
         <v>28</v>
       </c>
       <c r="E71" s="18" t="s">
+        <v>192</v>
+      </c>
+      <c r="F71" s="18" t="s">
         <v>193</v>
-      </c>
-      <c r="F71" s="18" t="s">
-        <v>194</v>
       </c>
       <c r="G71" s="27">
         <f>WORKDAY(總覽!$C$4,A71-1)</f>
@@ -4076,10 +4186,10 @@
         <v>28</v>
       </c>
       <c r="E72" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="F72" s="14" t="s">
         <v>195</v>
-      </c>
-      <c r="F72" s="14" t="s">
-        <v>196</v>
       </c>
       <c r="G72" s="26">
         <f>WORKDAY(總覽!$C$4,A72-1)</f>
@@ -4107,10 +4217,10 @@
         <v>28</v>
       </c>
       <c r="E73" s="18" t="s">
+        <v>196</v>
+      </c>
+      <c r="F73" s="18" t="s">
         <v>197</v>
-      </c>
-      <c r="F73" s="18" t="s">
-        <v>198</v>
       </c>
       <c r="G73" s="27">
         <f>WORKDAY(總覽!$C$4,A73-1)</f>
@@ -4138,10 +4248,10 @@
         <v>28</v>
       </c>
       <c r="E74" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="F74" s="18" t="s">
         <v>199</v>
-      </c>
-      <c r="F74" s="18" t="s">
-        <v>200</v>
       </c>
       <c r="G74" s="27">
         <f>WORKDAY(總覽!$C$4,A74-1)</f>
@@ -4169,10 +4279,10 @@
         <v>28</v>
       </c>
       <c r="E75" s="18" t="s">
+        <v>200</v>
+      </c>
+      <c r="F75" s="18" t="s">
         <v>201</v>
-      </c>
-      <c r="F75" s="18" t="s">
-        <v>202</v>
       </c>
       <c r="G75" s="27">
         <f>WORKDAY(總覽!$C$4,A75-1)</f>
@@ -4200,10 +4310,10 @@
         <v>28</v>
       </c>
       <c r="E76" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="F76" s="18" t="s">
         <v>203</v>
-      </c>
-      <c r="F76" s="18" t="s">
-        <v>204</v>
       </c>
       <c r="G76" s="27">
         <f>WORKDAY(總覽!$C$4,A76-1)</f>
@@ -4231,10 +4341,10 @@
         <v>28</v>
       </c>
       <c r="E77" s="14" t="s">
+        <v>204</v>
+      </c>
+      <c r="F77" s="14" t="s">
         <v>205</v>
-      </c>
-      <c r="F77" s="14" t="s">
-        <v>206</v>
       </c>
       <c r="G77" s="26">
         <f>WORKDAY(總覽!$C$4,A77-1)</f>
@@ -4262,10 +4372,10 @@
         <v>28</v>
       </c>
       <c r="E78" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="F78" s="18" t="s">
         <v>207</v>
-      </c>
-      <c r="F78" s="18" t="s">
-        <v>208</v>
       </c>
       <c r="G78" s="27">
         <f>WORKDAY(總覽!$C$4,A78-1)</f>
@@ -4293,10 +4403,10 @@
         <v>28</v>
       </c>
       <c r="E79" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="F79" s="18" t="s">
         <v>209</v>
-      </c>
-      <c r="F79" s="18" t="s">
-        <v>210</v>
       </c>
       <c r="G79" s="27">
         <f>WORKDAY(總覽!$C$4,A79-1)</f>
@@ -4324,10 +4434,10 @@
         <v>28</v>
       </c>
       <c r="E80" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="F80" s="18" t="s">
         <v>211</v>
-      </c>
-      <c r="F80" s="18" t="s">
-        <v>212</v>
       </c>
       <c r="G80" s="27">
         <f>WORKDAY(總覽!$C$4,A80-1)</f>
@@ -4355,10 +4465,10 @@
         <v>28</v>
       </c>
       <c r="E81" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="F81" s="18" t="s">
         <v>213</v>
-      </c>
-      <c r="F81" s="18" t="s">
-        <v>214</v>
       </c>
       <c r="G81" s="27">
         <f>WORKDAY(總覽!$C$4,A81-1)</f>
@@ -4386,10 +4496,10 @@
         <v>28</v>
       </c>
       <c r="E82" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="F82" s="14" t="s">
         <v>215</v>
-      </c>
-      <c r="F82" s="14" t="s">
-        <v>216</v>
       </c>
       <c r="G82" s="26">
         <f>WORKDAY(總覽!$C$4,A82-1)</f>
@@ -4417,10 +4527,10 @@
         <v>28</v>
       </c>
       <c r="E83" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="F83" s="18" t="s">
         <v>217</v>
-      </c>
-      <c r="F83" s="18" t="s">
-        <v>218</v>
       </c>
       <c r="G83" s="27">
         <f>WORKDAY(總覽!$C$4,A83-1)</f>
@@ -4448,10 +4558,10 @@
         <v>28</v>
       </c>
       <c r="E84" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="F84" s="18" t="s">
         <v>219</v>
-      </c>
-      <c r="F84" s="18" t="s">
-        <v>220</v>
       </c>
       <c r="G84" s="27">
         <f>WORKDAY(總覽!$C$4,A84-1)</f>
@@ -4479,10 +4589,10 @@
         <v>28</v>
       </c>
       <c r="E85" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="F85" s="18" t="s">
         <v>221</v>
-      </c>
-      <c r="F85" s="18" t="s">
-        <v>222</v>
       </c>
       <c r="G85" s="27">
         <f>WORKDAY(總覽!$C$4,A85-1)</f>
@@ -4510,10 +4620,10 @@
         <v>28</v>
       </c>
       <c r="E86" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="F86" s="18" t="s">
         <v>223</v>
-      </c>
-      <c r="F86" s="18" t="s">
-        <v>224</v>
       </c>
       <c r="G86" s="27">
         <f>WORKDAY(總覽!$C$4,A86-1)</f>
@@ -4541,10 +4651,10 @@
         <v>28</v>
       </c>
       <c r="E87" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="F87" s="14" t="s">
         <v>225</v>
-      </c>
-      <c r="F87" s="14" t="s">
-        <v>226</v>
       </c>
       <c r="G87" s="26">
         <f>WORKDAY(總覽!$C$4,A87-1)</f>
@@ -4572,10 +4682,10 @@
         <v>28</v>
       </c>
       <c r="E88" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="F88" s="18" t="s">
         <v>227</v>
-      </c>
-      <c r="F88" s="18" t="s">
-        <v>228</v>
       </c>
       <c r="G88" s="27">
         <f>WORKDAY(總覽!$C$4,A88-1)</f>
@@ -4603,10 +4713,10 @@
         <v>28</v>
       </c>
       <c r="E89" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="F89" s="18" t="s">
         <v>229</v>
-      </c>
-      <c r="F89" s="18" t="s">
-        <v>230</v>
       </c>
       <c r="G89" s="27">
         <f>WORKDAY(總覽!$C$4,A89-1)</f>
@@ -4634,10 +4744,10 @@
         <v>28</v>
       </c>
       <c r="E90" s="18" t="s">
+        <v>230</v>
+      </c>
+      <c r="F90" s="18" t="s">
         <v>231</v>
-      </c>
-      <c r="F90" s="18" t="s">
-        <v>232</v>
       </c>
       <c r="G90" s="27">
         <f>WORKDAY(總覽!$C$4,A90-1)</f>
@@ -4665,10 +4775,10 @@
         <v>28</v>
       </c>
       <c r="E91" s="18" t="s">
+        <v>232</v>
+      </c>
+      <c r="F91" s="18" t="s">
         <v>233</v>
-      </c>
-      <c r="F91" s="18" t="s">
-        <v>234</v>
       </c>
       <c r="G91" s="27">
         <f>WORKDAY(總覽!$C$4,A91-1)</f>
@@ -4696,10 +4806,10 @@
         <v>28</v>
       </c>
       <c r="E92" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="F92" s="14" t="s">
         <v>235</v>
-      </c>
-      <c r="F92" s="14" t="s">
-        <v>236</v>
       </c>
       <c r="G92" s="26">
         <f>WORKDAY(總覽!$C$4,A92-1)</f>
@@ -4727,10 +4837,10 @@
         <v>28</v>
       </c>
       <c r="E93" s="18" t="s">
+        <v>236</v>
+      </c>
+      <c r="F93" s="18" t="s">
         <v>237</v>
-      </c>
-      <c r="F93" s="18" t="s">
-        <v>238</v>
       </c>
       <c r="G93" s="27">
         <f>WORKDAY(總覽!$C$4,A93-1)</f>
@@ -4758,10 +4868,10 @@
         <v>28</v>
       </c>
       <c r="E94" s="18" t="s">
+        <v>238</v>
+      </c>
+      <c r="F94" s="18" t="s">
         <v>239</v>
-      </c>
-      <c r="F94" s="18" t="s">
-        <v>240</v>
       </c>
       <c r="G94" s="27">
         <f>WORKDAY(總覽!$C$4,A94-1)</f>
@@ -4789,10 +4899,10 @@
         <v>28</v>
       </c>
       <c r="E95" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="F95" s="18" t="s">
         <v>241</v>
-      </c>
-      <c r="F95" s="18" t="s">
-        <v>242</v>
       </c>
       <c r="G95" s="27">
         <f>WORKDAY(總覽!$C$4,A95-1)</f>
@@ -4820,10 +4930,10 @@
         <v>28</v>
       </c>
       <c r="E96" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="F96" s="18" t="s">
         <v>243</v>
-      </c>
-      <c r="F96" s="18" t="s">
-        <v>244</v>
       </c>
       <c r="G96" s="27">
         <f>WORKDAY(總覽!$C$4,A96-1)</f>
@@ -4851,10 +4961,10 @@
         <v>30</v>
       </c>
       <c r="E97" s="14" t="s">
+        <v>244</v>
+      </c>
+      <c r="F97" s="14" t="s">
         <v>245</v>
-      </c>
-      <c r="F97" s="14" t="s">
-        <v>246</v>
       </c>
       <c r="G97" s="26">
         <f>WORKDAY(總覽!$C$4,A97-1)</f>
@@ -4882,10 +4992,10 @@
         <v>30</v>
       </c>
       <c r="E98" s="18" t="s">
+        <v>246</v>
+      </c>
+      <c r="F98" s="18" t="s">
         <v>247</v>
-      </c>
-      <c r="F98" s="18" t="s">
-        <v>248</v>
       </c>
       <c r="G98" s="27">
         <f>WORKDAY(總覽!$C$4,A98-1)</f>
@@ -4913,10 +5023,10 @@
         <v>30</v>
       </c>
       <c r="E99" s="18" t="s">
+        <v>248</v>
+      </c>
+      <c r="F99" s="18" t="s">
         <v>249</v>
-      </c>
-      <c r="F99" s="18" t="s">
-        <v>250</v>
       </c>
       <c r="G99" s="27">
         <f>WORKDAY(總覽!$C$4,A99-1)</f>
@@ -4944,10 +5054,10 @@
         <v>30</v>
       </c>
       <c r="E100" s="18" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="F100" s="18" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G100" s="27">
         <f>WORKDAY(總覽!$C$4,A100-1)</f>
@@ -4975,10 +5085,10 @@
         <v>30</v>
       </c>
       <c r="E101" s="18" t="s">
+        <v>251</v>
+      </c>
+      <c r="F101" s="18" t="s">
         <v>252</v>
-      </c>
-      <c r="F101" s="18" t="s">
-        <v>253</v>
       </c>
       <c r="G101" s="27">
         <f>WORKDAY(總覽!$C$4,A101-1)</f>
@@ -5035,16 +5145,16 @@
         <v>14</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>45</v>
       </c>
       <c r="E1" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>255</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -5055,7 +5165,7 @@
         <v>16</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D2" s="19"/>
       <c r="E2" s="28"/>
@@ -5069,7 +5179,7 @@
         <v>16</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D3" s="19"/>
       <c r="E3" s="28"/>
@@ -5083,7 +5193,7 @@
         <v>18</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D4" s="19"/>
       <c r="E4" s="28"/>
@@ -5097,7 +5207,7 @@
         <v>18</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D5" s="19"/>
       <c r="E5" s="28"/>
@@ -5111,7 +5221,7 @@
         <v>20</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D6" s="19"/>
       <c r="E6" s="28"/>
@@ -5125,7 +5235,7 @@
         <v>20</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D7" s="19"/>
       <c r="E7" s="28"/>
@@ -5139,7 +5249,7 @@
         <v>20</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D8" s="19"/>
       <c r="E8" s="28"/>
@@ -5153,7 +5263,7 @@
         <v>22</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D9" s="19"/>
       <c r="E9" s="28"/>
@@ -5167,7 +5277,7 @@
         <v>22</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D10" s="19"/>
       <c r="E10" s="28"/>
@@ -5181,7 +5291,7 @@
         <v>24</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D11" s="19"/>
       <c r="E11" s="28"/>
@@ -5195,7 +5305,7 @@
         <v>24</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D12" s="19"/>
       <c r="E12" s="28"/>
@@ -5209,7 +5319,7 @@
         <v>26</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D13" s="19"/>
       <c r="E13" s="28"/>
@@ -5223,7 +5333,7 @@
         <v>26</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D14" s="19"/>
       <c r="E14" s="28"/>
@@ -5237,7 +5347,7 @@
         <v>28</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D15" s="19"/>
       <c r="E15" s="28"/>
@@ -5251,7 +5361,7 @@
         <v>28</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D16" s="19"/>
       <c r="E16" s="28"/>
@@ -5265,7 +5375,7 @@
         <v>28</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D17" s="19"/>
       <c r="E17" s="28"/>
@@ -5279,7 +5389,7 @@
         <v>28</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D18" s="19"/>
       <c r="E18" s="28"/>
@@ -5293,7 +5403,7 @@
         <v>28</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D19" s="19"/>
       <c r="E19" s="28"/>
@@ -5307,7 +5417,7 @@
         <v>28</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D20" s="19"/>
       <c r="E20" s="28"/>
@@ -5321,7 +5431,7 @@
         <v>30</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D21" s="19"/>
       <c r="E21" s="28"/>

</xml_diff>

<commit_message>
Add Day07 LINQ exercises
- Day07_LinQ: rewrite Day02 stats with LINQ (Count/Sum/Average/Max/Min),
  Where, Select, OrderByDescending/ThenBy, FirstOrDefault, Any, Contains, GroupBy
- Update progress sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/學習進度打卡表.xlsx
+++ b/學習進度打卡表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\林芯緹\Desktop\Learn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1469646-49B0-4071-93FB-5E1E22556B4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD79C2A-F2FC-4953-8526-4A13C57C98B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-135" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="總覽" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="281">
   <si>
     <t>C# .NET 學習進度打卡表</t>
   </si>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF(每日打卡!$H$2:$H$101,"✔")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="2:4">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C10" s="23">
         <f>IFERROR(C8/C9,0)</f>
-        <v>0.06</v>
+        <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="11" spans="2:4">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C11" s="24">
         <f>SUM(每日打卡!$J$2:$J$101)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="2:4">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="D18" s="11">
         <f>COUNTIFS(每日打卡!$D$2:$D$101,B18,每日打卡!$H$2:$H$101,"✔")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E18" s="11">
         <f>COUNTIF(每日打卡!$D$2:$D$101,B18)</f>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F18" s="12">
         <f t="shared" ref="F18:F25" si="0">IFERROR(D18/E18,0)</f>
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="19" spans="2:7">
@@ -2211,12 +2211,16 @@
         <f>WORKDAY(總覽!$C$4,A8-1)</f>
         <v>46301</v>
       </c>
-      <c r="H8" s="19"/>
+      <c r="H8" s="19" t="s">
+        <v>52</v>
+      </c>
       <c r="I8" s="17">
         <f>總覽!$C$5</f>
         <v>3.5</v>
       </c>
-      <c r="J8" s="19"/>
+      <c r="J8" s="19">
+        <v>2</v>
+      </c>
       <c r="K8" s="20"/>
     </row>
     <row r="9" spans="1:11">

</xml_diff>

<commit_message>
Add Day08 contacts validation and error handling
- Day08_Contacts: try/catch for blank names, nullable fixes (?? ""),
  ContactType enum with Enum.TryParse + IsDefined, CreatedAt DateTime
- Update study handoff notes and progress sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/學習進度打卡表.xlsx
+++ b/學習進度打卡表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\林芯緹\Desktop\Learn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD79C2A-F2FC-4953-8526-4A13C57C98B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B769C53A-3EFA-4C71-A1BB-CADAE70F15BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2625" yWindow="1005" windowWidth="26145" windowHeight="12750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="總覽" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="510" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="281">
   <si>
     <t>C# .NET 學習進度打卡表</t>
   </si>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF(每日打卡!$H$2:$H$101,"✔")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="2:4">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C10" s="23">
         <f>IFERROR(C8/C9,0)</f>
-        <v>7.0000000000000007E-2</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="11" spans="2:4">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C11" s="24">
         <f>SUM(每日打卡!$J$2:$J$101)</f>
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="2:4">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="D18" s="11">
         <f>COUNTIFS(每日打卡!$D$2:$D$101,B18,每日打卡!$H$2:$H$101,"✔")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E18" s="11">
         <f>COUNTIF(每日打卡!$D$2:$D$101,B18)</f>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F18" s="12">
         <f t="shared" ref="F18:F25" si="0">IFERROR(D18/E18,0)</f>
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="19" spans="2:7">
@@ -2246,12 +2246,16 @@
         <f>WORKDAY(總覽!$C$4,A9-1)</f>
         <v>46302</v>
       </c>
-      <c r="H9" s="19"/>
+      <c r="H9" s="19" t="s">
+        <v>52</v>
+      </c>
       <c r="I9" s="17">
         <f>總覽!$C$5</f>
         <v>3.5</v>
       </c>
-      <c r="J9" s="19"/>
+      <c r="J9" s="19">
+        <v>2</v>
+      </c>
       <c r="K9" s="20"/>
     </row>
     <row r="10" spans="1:11">

</xml_diff>

<commit_message>
Add Day09 contacts JSON persistence and async save
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/學習進度打卡表.xlsx
+++ b/學習進度打卡表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\林芯緹\Desktop\Learn\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B769C53A-3EFA-4C71-A1BB-CADAE70F15BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C887DE6C-95F7-4943-A042-EA3A93770DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2625" yWindow="1005" windowWidth="26145" windowHeight="12750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2235" yWindow="1500" windowWidth="26145" windowHeight="12750" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="總覽" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="281">
   <si>
     <t>C# .NET 學習進度打卡表</t>
   </si>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C8" s="7">
         <f>COUNTIF(每日打卡!$H$2:$H$101,"✔")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="2:4">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="C10" s="23">
         <f>IFERROR(C8/C9,0)</f>
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="11" spans="2:4">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="C11" s="24">
         <f>SUM(每日打卡!$J$2:$J$101)</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="2:4">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="D18" s="11">
         <f>COUNTIFS(每日打卡!$D$2:$D$101,B18,每日打卡!$H$2:$H$101,"✔")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E18" s="11">
         <f>COUNTIF(每日打卡!$D$2:$D$101,B18)</f>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="F18" s="12">
         <f t="shared" ref="F18:F25" si="0">IFERROR(D18/E18,0)</f>
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="19" spans="2:7">
@@ -2281,12 +2281,16 @@
         <f>WORKDAY(總覽!$C$4,A10-1)</f>
         <v>46303</v>
       </c>
-      <c r="H10" s="19"/>
+      <c r="H10" s="19" t="s">
+        <v>52</v>
+      </c>
       <c r="I10" s="17">
         <f>總覽!$C$5</f>
         <v>3.5</v>
       </c>
-      <c r="J10" s="19"/>
+      <c r="J10" s="19">
+        <v>2</v>
+      </c>
       <c r="K10" s="20"/>
     </row>
     <row r="11" spans="1:11">

</xml_diff>